<commit_message>
Add Obsidian project notes
</commit_message>
<xml_diff>
--- a/data/processed/my_album_status.xlsx
+++ b/data/processed/my_album_status.xlsx
@@ -2537,7 +2537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr filterMode="1"/>
+  <sheetPr/>
   <dimension ref="A1:M133"/>
   <sheetFormatPr defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
@@ -2597,7 +2597,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" hidden="1" spans="1:13">
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -2635,7 +2635,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" hidden="1" spans="1:13">
+    <row r="3" spans="1:13">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -2711,7 +2711,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" hidden="1" spans="1:13">
+    <row r="5" spans="1:13">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -2787,7 +2787,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" hidden="1" spans="1:13">
+    <row r="7" spans="1:13">
       <c r="A7" t="s">
         <v>38</v>
       </c>
@@ -2863,7 +2863,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" hidden="1" spans="1:13">
+    <row r="9" spans="1:13">
       <c r="A9" t="s">
         <v>46</v>
       </c>
@@ -2901,7 +2901,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" hidden="1" spans="1:13">
+    <row r="10" spans="1:13">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -2939,7 +2939,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" hidden="1" spans="1:13">
+    <row r="11" spans="1:13">
       <c r="A11" t="s">
         <v>53</v>
       </c>
@@ -3015,7 +3015,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="13" hidden="1" spans="1:13">
+    <row r="13" spans="1:13">
       <c r="A13" t="s">
         <v>61</v>
       </c>
@@ -3091,7 +3091,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" hidden="1" spans="1:13">
+    <row r="15" spans="1:13">
       <c r="A15" t="s">
         <v>69</v>
       </c>
@@ -3231,7 +3231,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="19" hidden="1" spans="1:12">
+    <row r="19" spans="1:12">
       <c r="A19" t="s">
         <v>85</v>
       </c>
@@ -3307,7 +3307,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" hidden="1" spans="1:12">
+    <row r="21" spans="1:12">
       <c r="A21" t="s">
         <v>93</v>
       </c>
@@ -3345,7 +3345,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" hidden="1" spans="1:12">
+    <row r="22" spans="1:12">
       <c r="A22" t="s">
         <v>97</v>
       </c>
@@ -3383,7 +3383,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="23" hidden="1" spans="1:12">
+    <row r="23" spans="1:12">
       <c r="A23" t="s">
         <v>73</v>
       </c>
@@ -3459,7 +3459,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" hidden="1" spans="1:12">
+    <row r="25" spans="1:12">
       <c r="A25" t="s">
         <v>108</v>
       </c>
@@ -3535,7 +3535,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" hidden="1" spans="1:12">
+    <row r="27" spans="1:12">
       <c r="A27" t="s">
         <v>116</v>
       </c>
@@ -3573,7 +3573,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="28" hidden="1" spans="1:12">
+    <row r="28" spans="1:12">
       <c r="A28" t="s">
         <v>53</v>
       </c>
@@ -3637,7 +3637,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="30" hidden="1" spans="1:12">
+    <row r="30" spans="1:12">
       <c r="A30" t="s">
         <v>125</v>
       </c>
@@ -3675,7 +3675,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="31" hidden="1" spans="1:12">
+    <row r="31" spans="1:12">
       <c r="A31" t="s">
         <v>129</v>
       </c>
@@ -3710,7 +3710,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="32" hidden="1" spans="1:12">
+    <row r="32" spans="1:12">
       <c r="A32" t="s">
         <v>38</v>
       </c>
@@ -3786,7 +3786,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="34" hidden="1" spans="1:12">
+    <row r="34" spans="1:12">
       <c r="A34" t="s">
         <v>46</v>
       </c>
@@ -3824,7 +3824,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="35" hidden="1" spans="1:12">
+    <row r="35" spans="1:12">
       <c r="A35" t="s">
         <v>145</v>
       </c>
@@ -3935,7 +3935,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="38" hidden="1" spans="1:12">
+    <row r="38" spans="1:12">
       <c r="A38" t="s">
         <v>157</v>
       </c>
@@ -3970,7 +3970,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="39" hidden="1" spans="1:12">
+    <row r="39" spans="1:12">
       <c r="A39" t="s">
         <v>161</v>
       </c>
@@ -3996,7 +3996,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" hidden="1" spans="1:12">
+    <row r="40" spans="1:12">
       <c r="A40" t="s">
         <v>163</v>
       </c>
@@ -4110,7 +4110,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="43" hidden="1" spans="1:12">
+    <row r="43" spans="1:12">
       <c r="A43" t="s">
         <v>175</v>
       </c>
@@ -4145,7 +4145,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="44" hidden="1" spans="1:12">
+    <row r="44" spans="1:12">
       <c r="A44" t="s">
         <v>179</v>
       </c>
@@ -4183,7 +4183,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="45" hidden="1" spans="1:12">
+    <row r="45" spans="1:12">
       <c r="A45" t="s">
         <v>183</v>
       </c>
@@ -4259,7 +4259,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="47" hidden="1" spans="1:12">
+    <row r="47" spans="1:12">
       <c r="A47" t="s">
         <v>104</v>
       </c>
@@ -4297,7 +4297,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="48" hidden="1" spans="1:12">
+    <row r="48" spans="1:12">
       <c r="A48" t="s">
         <v>194</v>
       </c>
@@ -4373,7 +4373,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="50" hidden="1" spans="1:12">
+    <row r="50" spans="1:12">
       <c r="A50" t="s">
         <v>202</v>
       </c>
@@ -4399,7 +4399,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="51" hidden="1" spans="1:12">
+    <row r="51" spans="1:12">
       <c r="A51" t="s">
         <v>204</v>
       </c>
@@ -4451,7 +4451,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="53" hidden="1" spans="1:12">
+    <row r="53" spans="1:12">
       <c r="A53" t="s">
         <v>208</v>
       </c>
@@ -4486,7 +4486,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="54" hidden="1" spans="1:12">
+    <row r="54" spans="1:12">
       <c r="A54" t="s">
         <v>212</v>
       </c>
@@ -4512,7 +4512,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="55" hidden="1" spans="1:12">
+    <row r="55" spans="1:12">
       <c r="A55" t="s">
         <v>214</v>
       </c>
@@ -4585,7 +4585,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="57" hidden="1" spans="1:12">
+    <row r="57" spans="1:12">
       <c r="A57" t="s">
         <v>222</v>
       </c>
@@ -4637,7 +4637,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="59" hidden="1" spans="1:12">
+    <row r="59" spans="1:12">
       <c r="A59" t="s">
         <v>42</v>
       </c>
@@ -4710,7 +4710,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="61" hidden="1" spans="1:12">
+    <row r="61" spans="1:12">
       <c r="A61" t="s">
         <v>73</v>
       </c>
@@ -4736,7 +4736,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="62" hidden="1" spans="1:12">
+    <row r="62" spans="1:12">
       <c r="A62" t="s">
         <v>234</v>
       </c>
@@ -4771,7 +4771,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="63" hidden="1" spans="1:12">
+    <row r="63" spans="1:12">
       <c r="A63" t="s">
         <v>104</v>
       </c>
@@ -4885,7 +4885,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="66" hidden="1" spans="1:12">
+    <row r="66" spans="1:12">
       <c r="A66" t="s">
         <v>249</v>
       </c>
@@ -4920,7 +4920,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="67" hidden="1" spans="1:12">
+    <row r="67" spans="1:12">
       <c r="A67" t="s">
         <v>253</v>
       </c>
@@ -4946,7 +4946,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="68" hidden="1" spans="1:12">
+    <row r="68" spans="1:12">
       <c r="A68" t="s">
         <v>255</v>
       </c>
@@ -5019,7 +5019,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="70" hidden="1" spans="1:12">
+    <row r="70" spans="1:12">
       <c r="A70" t="s">
         <v>73</v>
       </c>
@@ -5045,7 +5045,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="71" hidden="1" spans="1:12">
+    <row r="71" spans="1:12">
       <c r="A71" t="s">
         <v>264</v>
       </c>
@@ -5080,7 +5080,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="72" hidden="1" spans="1:12">
+    <row r="72" spans="1:12">
       <c r="A72" t="s">
         <v>149</v>
       </c>
@@ -5118,7 +5118,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="73" hidden="1" spans="1:12">
+    <row r="73" spans="1:12">
       <c r="A73" t="s">
         <v>85</v>
       </c>
@@ -5156,7 +5156,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="74" hidden="1" spans="1:12">
+    <row r="74" spans="1:12">
       <c r="A74" t="s">
         <v>42</v>
       </c>
@@ -5194,7 +5194,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="75" hidden="1" spans="1:12">
+    <row r="75" spans="1:12">
       <c r="A75" t="s">
         <v>277</v>
       </c>
@@ -5232,7 +5232,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="76" hidden="1" spans="1:12">
+    <row r="76" spans="1:12">
       <c r="A76" t="s">
         <v>281</v>
       </c>
@@ -5331,7 +5331,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="79" hidden="1" spans="1:12">
+    <row r="79" spans="1:12">
       <c r="A79" t="s">
         <v>291</v>
       </c>
@@ -5392,7 +5392,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="81" hidden="1" spans="1:12">
+    <row r="81" spans="1:12">
       <c r="A81" t="s">
         <v>171</v>
       </c>
@@ -5418,7 +5418,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="82" hidden="1" spans="1:12">
+    <row r="82" spans="1:12">
       <c r="A82" t="s">
         <v>297</v>
       </c>
@@ -5453,7 +5453,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="83" hidden="1" spans="1:12">
+    <row r="83" spans="1:12">
       <c r="A83" t="s">
         <v>301</v>
       </c>
@@ -5491,7 +5491,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="84" hidden="1" spans="1:12">
+    <row r="84" spans="1:12">
       <c r="A84" t="s">
         <v>305</v>
       </c>
@@ -5517,7 +5517,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="85" hidden="1" spans="1:12">
+    <row r="85" spans="1:12">
       <c r="A85" t="s">
         <v>307</v>
       </c>
@@ -5555,7 +5555,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="86" hidden="1" spans="1:12">
+    <row r="86" spans="1:12">
       <c r="A86" t="s">
         <v>311</v>
       </c>
@@ -5683,7 +5683,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="90" hidden="1" spans="1:12">
+    <row r="90" spans="1:12">
       <c r="A90" t="s">
         <v>321</v>
       </c>
@@ -5721,7 +5721,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="91" hidden="1" spans="1:12">
+    <row r="91" spans="1:12">
       <c r="A91" t="s">
         <v>149</v>
       </c>
@@ -5829,7 +5829,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="94" hidden="1" spans="1:12">
+    <row r="94" spans="1:12">
       <c r="A94" t="s">
         <v>336</v>
       </c>
@@ -5855,7 +5855,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="95" hidden="1" spans="1:12">
+    <row r="95" spans="1:12">
       <c r="A95" t="s">
         <v>287</v>
       </c>
@@ -5893,7 +5893,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="96" hidden="1" spans="1:12">
+    <row r="96" spans="1:12">
       <c r="A96" t="s">
         <v>341</v>
       </c>
@@ -5928,7 +5928,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="97" hidden="1" spans="1:12">
+    <row r="97" spans="1:12">
       <c r="A97" t="s">
         <v>108</v>
       </c>
@@ -5954,7 +5954,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="98" hidden="1" spans="1:12">
+    <row r="98" spans="1:12">
       <c r="A98" t="s">
         <v>346</v>
       </c>
@@ -6030,7 +6030,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="100" hidden="1" spans="1:12">
+    <row r="100" spans="1:12">
       <c r="A100" t="s">
         <v>346</v>
       </c>
@@ -6065,7 +6065,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="101" hidden="1" spans="1:12">
+    <row r="101" spans="1:12">
       <c r="A101" t="s">
         <v>357</v>
       </c>
@@ -6091,7 +6091,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="102" hidden="1" spans="1:12">
+    <row r="102" spans="1:12">
       <c r="A102" t="s">
         <v>359</v>
       </c>
@@ -6126,7 +6126,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="103" hidden="1" spans="1:12">
+    <row r="103" spans="1:12">
       <c r="A103" t="s">
         <v>363</v>
       </c>
@@ -6152,7 +6152,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="104" hidden="1" spans="1:12">
+    <row r="104" spans="1:12">
       <c r="A104" t="s">
         <v>365</v>
       </c>
@@ -6187,7 +6187,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="105" hidden="1" spans="1:12">
+    <row r="105" spans="1:12">
       <c r="A105" t="s">
         <v>369</v>
       </c>
@@ -6225,7 +6225,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="106" hidden="1" spans="1:12">
+    <row r="106" spans="1:12">
       <c r="A106" t="s">
         <v>373</v>
       </c>
@@ -6260,7 +6260,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="107" hidden="1" spans="1:12">
+    <row r="107" spans="1:12">
       <c r="A107" t="s">
         <v>377</v>
       </c>
@@ -6286,7 +6286,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="108" hidden="1" spans="1:12">
+    <row r="108" spans="1:12">
       <c r="A108" t="s">
         <v>378</v>
       </c>
@@ -6321,7 +6321,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="109" hidden="1" spans="1:12">
+    <row r="109" spans="1:12">
       <c r="A109" t="s">
         <v>85</v>
       </c>
@@ -6359,7 +6359,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="110" hidden="1" spans="1:12">
+    <row r="110" spans="1:12">
       <c r="A110" t="s">
         <v>204</v>
       </c>
@@ -6394,7 +6394,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="111" hidden="1" spans="1:12">
+    <row r="111" spans="1:12">
       <c r="A111" t="s">
         <v>187</v>
       </c>
@@ -6432,7 +6432,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="112" hidden="1" spans="1:12">
+    <row r="112" spans="1:12">
       <c r="A112" t="s">
         <v>391</v>
       </c>
@@ -6505,7 +6505,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="114" hidden="1" spans="1:12">
+    <row r="114" spans="1:12">
       <c r="A114" t="s">
         <v>399</v>
       </c>
@@ -6531,7 +6531,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="115" hidden="1" spans="1:12">
+    <row r="115" spans="1:12">
       <c r="A115" t="s">
         <v>198</v>
       </c>
@@ -6566,7 +6566,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="116" hidden="1" spans="1:12">
+    <row r="116" spans="1:12">
       <c r="A116" t="s">
         <v>321</v>
       </c>
@@ -6592,7 +6592,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="117" hidden="1" spans="1:12">
+    <row r="117" spans="1:12">
       <c r="A117" t="s">
         <v>391</v>
       </c>
@@ -6627,7 +6627,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="118" hidden="1" spans="1:12">
+    <row r="118" spans="1:12">
       <c r="A118" t="s">
         <v>198</v>
       </c>
@@ -6665,7 +6665,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="119" hidden="1" spans="1:12">
+    <row r="119" spans="1:12">
       <c r="A119" t="s">
         <v>321</v>
       </c>
@@ -6691,7 +6691,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="120" hidden="1" spans="1:12">
+    <row r="120" spans="1:12">
       <c r="A120" t="s">
         <v>412</v>
       </c>
@@ -6726,7 +6726,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="121" hidden="1" spans="1:12">
+    <row r="121" spans="1:12">
       <c r="A121" t="s">
         <v>416</v>
       </c>
@@ -6764,7 +6764,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="122" hidden="1" spans="1:12">
+    <row r="122" spans="1:12">
       <c r="A122" t="s">
         <v>420</v>
       </c>
@@ -6799,7 +6799,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="123" hidden="1" spans="1:12">
+    <row r="123" spans="1:12">
       <c r="A123" t="s">
         <v>424</v>
       </c>
@@ -6834,7 +6834,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="124" hidden="1" spans="1:12">
+    <row r="124" spans="1:12">
       <c r="A124" t="s">
         <v>253</v>
       </c>
@@ -6860,7 +6860,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="125" hidden="1" spans="1:12">
+    <row r="125" spans="1:12">
       <c r="A125" t="s">
         <v>429</v>
       </c>
@@ -6959,7 +6959,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="128" hidden="1" spans="1:12">
+    <row r="128" spans="1:12">
       <c r="A128" t="s">
         <v>439</v>
       </c>
@@ -6985,7 +6985,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="129" hidden="1" spans="1:12">
+    <row r="129" spans="1:12">
       <c r="A129" t="s">
         <v>441</v>
       </c>
@@ -7046,7 +7046,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="131" hidden="1" spans="1:12">
+    <row r="131" spans="1:12">
       <c r="A131" t="s">
         <v>108</v>
       </c>
@@ -7072,7 +7072,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="132" hidden="1" spans="1:12">
+    <row r="132" spans="1:12">
       <c r="A132" t="s">
         <v>447</v>
       </c>
@@ -7107,7 +7107,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="133" hidden="1" spans="1:12">
+    <row r="133" spans="1:12">
       <c r="A133" t="s">
         <v>81</v>
       </c>
@@ -7135,13 +7135,6 @@
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:M133" etc:filterBottomFollowUsedRange="0">
-    <filterColumn colId="11">
-      <filters>
-        <filter val="low"/>
-        <filter val="high"/>
-        <filter val="medium"/>
-      </filters>
-    </filterColumn>
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>